<commit_message>
feat: update data bal tembakau tanggal 5 Oktober 2026 (11 bal, 477.0 kg, No Gud 2100-2188), sync Supabase, update rekap excel, dan bump cache version v=8.1
</commit_message>
<xml_diff>
--- a/Buku Grade Induk Urut Barkot/_REKAP_DAFTAR_PRINT_SEMUA_TANGGAL.xlsx
+++ b/Buku Grade Induk Urut Barkot/_REKAP_DAFTAR_PRINT_SEMUA_TANGGAL.xlsx
@@ -505,7 +505,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr fitToPage="1"/>
   </sheetPr>
-  <dimension ref="A1:H46"/>
+  <dimension ref="A1:H47"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="5" customWidth="1" min="1" max="1"/>
@@ -2086,30 +2086,66 @@
         </is>
       </c>
     </row>
-    <row r="46" ht="22" customHeight="1">
-      <c r="A46" s="3" t="inlineStr">
+    <row r="46" ht="18" customHeight="1">
+      <c r="A46" s="4" t="n">
+        <v>43</v>
+      </c>
+      <c r="B46" s="4" t="inlineStr">
+        <is>
+          <t>2026-10-05</t>
+        </is>
+      </c>
+      <c r="C46" s="4" t="inlineStr">
+        <is>
+          <t>SENIN</t>
+        </is>
+      </c>
+      <c r="D46" s="5" t="n">
+        <v>11</v>
+      </c>
+      <c r="E46" s="6" t="n">
+        <v>477</v>
+      </c>
+      <c r="F46" s="4" t="inlineStr">
+        <is>
+          <t>383371 s/d 578236</t>
+        </is>
+      </c>
+      <c r="G46" s="4" t="inlineStr">
+        <is>
+          <t>No. Gud 2100 - 2188</t>
+        </is>
+      </c>
+      <c r="H46" s="7" t="inlineStr">
+        <is>
+          <t>buku_grade_induk_2026-10-05_tgl_05_okt_urut_barkot.xlsx</t>
+        </is>
+      </c>
+    </row>
+    <row r="47" ht="22" customHeight="1">
+      <c r="A47" s="3" t="inlineStr">
         <is>
           <t>TOTAL KESELURUHAN</t>
         </is>
       </c>
-      <c r="B46" s="12" t="n"/>
-      <c r="C46" s="12" t="n"/>
-      <c r="D46" s="13">
-        <f>SUM(D4:D45)</f>
+      <c r="B47" s="12" t="n"/>
+      <c r="C47" s="12" t="n"/>
+      <c r="D47" s="13">
+        <f>SUM(D4:D46)</f>
         <v/>
       </c>
-      <c r="E46" s="14">
-        <f>SUM(E4:E45)</f>
+      <c r="E47" s="14">
+        <f>SUM(E4:E46)</f>
         <v/>
       </c>
-      <c r="F46" s="12" t="n"/>
-      <c r="G46" s="12" t="n"/>
-      <c r="H46" s="12" t="n"/>
+      <c r="F47" s="12" t="n"/>
+      <c r="G47" s="12" t="n"/>
+      <c r="H47" s="12" t="n"/>
     </row>
   </sheetData>
   <mergeCells count="3">
-    <mergeCell ref="A46:C46"/>
     <mergeCell ref="A2:H2"/>
+    <mergeCell ref="A47:C47"/>
     <mergeCell ref="A1:H1"/>
   </mergeCells>
   <printOptions horizontalCentered="1"/>

</xml_diff>

<commit_message>
feat: update data bal tembakau tanggal 6 Oktober 2026 (36 bal, 1504.0 kg, No Gud 2189-2224), sync Supabase, update rekap excel, dan bump cache version v=8.2
</commit_message>
<xml_diff>
--- a/Buku Grade Induk Urut Barkot/_REKAP_DAFTAR_PRINT_SEMUA_TANGGAL.xlsx
+++ b/Buku Grade Induk Urut Barkot/_REKAP_DAFTAR_PRINT_SEMUA_TANGGAL.xlsx
@@ -505,7 +505,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr fitToPage="1"/>
   </sheetPr>
-  <dimension ref="A1:H47"/>
+  <dimension ref="A1:H48"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="5" customWidth="1" min="1" max="1"/>
@@ -2122,30 +2122,66 @@
         </is>
       </c>
     </row>
-    <row r="47" ht="22" customHeight="1">
-      <c r="A47" s="3" t="inlineStr">
+    <row r="47" ht="18" customHeight="1">
+      <c r="A47" s="8" t="n">
+        <v>44</v>
+      </c>
+      <c r="B47" s="8" t="inlineStr">
+        <is>
+          <t>2026-10-06</t>
+        </is>
+      </c>
+      <c r="C47" s="8" t="inlineStr">
+        <is>
+          <t>SELASA</t>
+        </is>
+      </c>
+      <c r="D47" s="9" t="n">
+        <v>36</v>
+      </c>
+      <c r="E47" s="10" t="n">
+        <v>1504</v>
+      </c>
+      <c r="F47" s="8" t="inlineStr">
+        <is>
+          <t>383386 s/d 578616</t>
+        </is>
+      </c>
+      <c r="G47" s="8" t="inlineStr">
+        <is>
+          <t>No. Gud 2189 - 2224</t>
+        </is>
+      </c>
+      <c r="H47" s="11" t="inlineStr">
+        <is>
+          <t>buku_grade_induk_2026-10-06_tgl_06_okt_urut_barkot.xlsx</t>
+        </is>
+      </c>
+    </row>
+    <row r="48" ht="22" customHeight="1">
+      <c r="A48" s="3" t="inlineStr">
         <is>
           <t>TOTAL KESELURUHAN</t>
         </is>
       </c>
-      <c r="B47" s="12" t="n"/>
-      <c r="C47" s="12" t="n"/>
-      <c r="D47" s="13">
-        <f>SUM(D4:D46)</f>
+      <c r="B48" s="12" t="n"/>
+      <c r="C48" s="12" t="n"/>
+      <c r="D48" s="13">
+        <f>SUM(D4:D47)</f>
         <v/>
       </c>
-      <c r="E47" s="14">
-        <f>SUM(E4:E46)</f>
+      <c r="E48" s="14">
+        <f>SUM(E4:E47)</f>
         <v/>
       </c>
-      <c r="F47" s="12" t="n"/>
-      <c r="G47" s="12" t="n"/>
-      <c r="H47" s="12" t="n"/>
+      <c r="F48" s="12" t="n"/>
+      <c r="G48" s="12" t="n"/>
+      <c r="H48" s="12" t="n"/>
     </row>
   </sheetData>
   <mergeCells count="3">
+    <mergeCell ref="A48:C48"/>
     <mergeCell ref="A2:H2"/>
-    <mergeCell ref="A47:C47"/>
     <mergeCell ref="A1:H1"/>
   </mergeCells>
   <printOptions horizontalCentered="1"/>

</xml_diff>

<commit_message>
feat: update data bal tembakau tanggal 8 Oktober 2026 (29 bal, 1213.0 kg, No Gud 2173-2265), sync Supabase, update rekap excel, dan bump cache version v=8.3
</commit_message>
<xml_diff>
--- a/Buku Grade Induk Urut Barkot/_REKAP_DAFTAR_PRINT_SEMUA_TANGGAL.xlsx
+++ b/Buku Grade Induk Urut Barkot/_REKAP_DAFTAR_PRINT_SEMUA_TANGGAL.xlsx
@@ -505,7 +505,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr fitToPage="1"/>
   </sheetPr>
-  <dimension ref="A1:H48"/>
+  <dimension ref="A1:H49"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="5" customWidth="1" min="1" max="1"/>
@@ -2158,30 +2158,66 @@
         </is>
       </c>
     </row>
-    <row r="48" ht="22" customHeight="1">
-      <c r="A48" s="3" t="inlineStr">
+    <row r="48" ht="18" customHeight="1">
+      <c r="A48" s="4" t="n">
+        <v>45</v>
+      </c>
+      <c r="B48" s="4" t="inlineStr">
+        <is>
+          <t>2026-10-08</t>
+        </is>
+      </c>
+      <c r="C48" s="4" t="inlineStr">
+        <is>
+          <t>KAMIS</t>
+        </is>
+      </c>
+      <c r="D48" s="5" t="n">
+        <v>29</v>
+      </c>
+      <c r="E48" s="6" t="n">
+        <v>1213</v>
+      </c>
+      <c r="F48" s="4" t="inlineStr">
+        <is>
+          <t>578995 s/d 579804</t>
+        </is>
+      </c>
+      <c r="G48" s="4" t="inlineStr">
+        <is>
+          <t>No. Gud 2173 - 2265</t>
+        </is>
+      </c>
+      <c r="H48" s="7" t="inlineStr">
+        <is>
+          <t>buku_grade_induk_2026-10-08_tgl_08_okt_urut_barkot.xlsx</t>
+        </is>
+      </c>
+    </row>
+    <row r="49" ht="22" customHeight="1">
+      <c r="A49" s="3" t="inlineStr">
         <is>
           <t>TOTAL KESELURUHAN</t>
         </is>
       </c>
-      <c r="B48" s="12" t="n"/>
-      <c r="C48" s="12" t="n"/>
-      <c r="D48" s="13">
-        <f>SUM(D4:D47)</f>
+      <c r="B49" s="12" t="n"/>
+      <c r="C49" s="12" t="n"/>
+      <c r="D49" s="13">
+        <f>SUM(D4:D48)</f>
         <v/>
       </c>
-      <c r="E48" s="14">
-        <f>SUM(E4:E47)</f>
+      <c r="E49" s="14">
+        <f>SUM(E4:E48)</f>
         <v/>
       </c>
-      <c r="F48" s="12" t="n"/>
-      <c r="G48" s="12" t="n"/>
-      <c r="H48" s="12" t="n"/>
+      <c r="F49" s="12" t="n"/>
+      <c r="G49" s="12" t="n"/>
+      <c r="H49" s="12" t="n"/>
     </row>
   </sheetData>
   <mergeCells count="3">
-    <mergeCell ref="A48:C48"/>
     <mergeCell ref="A2:H2"/>
+    <mergeCell ref="A49:C49"/>
     <mergeCell ref="A1:H1"/>
   </mergeCells>
   <printOptions horizontalCentered="1"/>

</xml_diff>